<commit_message>
add feature for post/put event to event and delete event and uts format
</commit_message>
<xml_diff>
--- a/sample-format/dataElements_form_name_translations_with_object_property.xlsx
+++ b/sample-format/dataElements_form_name_translations_with_object_property.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\gitHub_source_code\excel_to_Json_Converter_angularJS\sample-format\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA72CEAB-BDB2-4FE3-9579-AE83BDE5D78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD96523E-B998-4500-AF34-F8EA55BD3C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2802" uniqueCount="1072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2806" uniqueCount="1076">
   <si>
     <t>property</t>
   </si>
@@ -3251,6 +3251,18 @@
   </si>
   <si>
     <t>tet</t>
+  </si>
+  <si>
+    <t>Hindi</t>
+  </si>
+  <si>
+    <t>hi</t>
+  </si>
+  <si>
+    <t>Nepali</t>
+  </si>
+  <si>
+    <t>ne</t>
   </si>
 </sst>
 </file>
@@ -3325,9 +3337,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3365,7 +3377,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3471,7 +3483,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3613,7 +3625,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3818,6 +3830,12 @@
       <c r="E8" t="s">
         <v>1047</v>
       </c>
+      <c r="G8" s="2" t="s">
+        <v>1072</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>1073</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
@@ -3834,6 +3852,12 @@
       </c>
       <c r="E9" t="s">
         <v>1053</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>1075</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -13427,12 +13451,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010064994C001712374395B345EB88ED991F" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c1a62579524e26006c6d5335831b55c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f9770305-a86c-4dd4-a8e3-5283c3e6bf99" xmlns:ns3="3f48127a-ff27-4c8f-88c3-e54b29f41588" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="658091719f3253a39288b5ed2add5a7b" ns2:_="" ns3:_="">
     <xsd:import namespace="f9770305-a86c-4dd4-a8e3-5283c3e6bf99"/>
@@ -13629,6 +13647,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -13639,15 +13663,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACBAC26C-ABD4-4796-8551-545E34A88729}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E76993AC-6818-4630-B1D6-F654BE5E03B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13666,6 +13681,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACBAC26C-ABD4-4796-8551-545E34A88729}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18A4371F-7DC5-4CF4-A869-E47776CCD6EB}">
   <ds:schemaRefs>

</xml_diff>